<commit_message>
r622: the common Trick sheet rebuilt on an audit of the current code
TRICKS_COMMON.xlsx / .csv now carry measurements from a Trick audit of
this code (tools/sim/out/trick-audit-r622.*: card ladder scoring, 6 deals
x 40 grids, 204 loadouts), not the r606 audit r620 shipped with. What moved
since: On the Edge pays per edge card (share 0.61 -> 1.94, fires 23% ->
76%), Aftershock pays now that two pairs read as a Two Pair (0.0 -> 0.42),
Kindling and Echoes read lower (1.33 -> 0.76, 1.68 -> 1.12). The outliers
are unchanged: Unsummit 3.94, Combo Score 3.19, Magician 2.68 times the
average Trick; Night Owl, Enriched and Tidal Forces barely fire for the
bot (it plays few flushes and plays through the round at one pace).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DfYx6rMENmrcJVZ5fpmg9G
</commit_message>
<xml_diff>
--- a/TRICKS_COMMON.xlsx
+++ b/TRICKS_COMMON.xlsx
@@ -641,7 +641,7 @@
         <v/>
       </c>
       <c r="K2" s="5" t="n">
-        <v>0.87</v>
+        <v>0.84</v>
       </c>
       <c r="L2" s="5" t="n">
         <v>1.36</v>
@@ -706,7 +706,7 @@
         <v/>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="L3" s="5" t="n">
         <v>1.23</v>
@@ -771,17 +771,17 @@
         <v/>
       </c>
       <c r="K4" s="5" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>1</v>
+        <v>1.18</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Barely pays</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr"/>
@@ -903,7 +903,7 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr"/>
@@ -954,7 +954,7 @@
         <v/>
       </c>
       <c r="K7" s="5" t="n">
-        <v>4.07</v>
+        <v>3.94</v>
       </c>
       <c r="L7" s="5" t="n">
         <v>2.67</v>
@@ -1019,7 +1019,7 @@
         <v/>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
       <c r="L8" s="5" t="n">
         <v>1.55</v>
@@ -1084,7 +1084,7 @@
         <v/>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="L9" s="5" t="n">
         <v>1.07</v>
@@ -1145,7 +1145,7 @@
         <v/>
       </c>
       <c r="K10" s="5" t="n">
-        <v>0.51</v>
+        <v>0.48</v>
       </c>
       <c r="L10" s="5" t="n">
         <v>1.21</v>
@@ -1210,7 +1210,7 @@
         <v/>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="L11" s="5" t="n">
         <v>1.33</v>
@@ -1304,7 +1304,7 @@
         <v/>
       </c>
       <c r="K13" s="5" t="n">
-        <v>1.16</v>
+        <v>1.12</v>
       </c>
       <c r="L13" s="5" t="n">
         <v>1.48</v>
@@ -1369,7 +1369,7 @@
         <v/>
       </c>
       <c r="K14" s="5" t="n">
-        <v>1.56</v>
+        <v>1.51</v>
       </c>
       <c r="L14" s="5" t="n">
         <v>1.64</v>
@@ -1671,7 +1671,7 @@
         <v/>
       </c>
       <c r="K20" s="5" t="n">
-        <v>1.12</v>
+        <v>1.09</v>
       </c>
       <c r="L20" s="5" t="n">
         <v>1.46</v>
@@ -1769,13 +1769,13 @@
         <v/>
       </c>
       <c r="K22" s="5" t="n">
-        <v>1.33</v>
+        <v>0.76</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>1.55</v>
+        <v>1.32</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
@@ -1825,17 +1825,17 @@
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="5" t="n"/>
       <c r="K23" s="5" t="n">
-        <v>1.68</v>
+        <v>1.12</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>1.69</v>
+        <v>1.48</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr"/>
@@ -1886,7 +1886,7 @@
         <v/>
       </c>
       <c r="K24" s="5" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="L24" s="5" t="n">
         <v>1.2</v>
@@ -1947,7 +1947,7 @@
         <v/>
       </c>
       <c r="K25" s="5" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="L25" s="5" t="n">
         <v>1.18</v>
@@ -2011,7 +2011,7 @@
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="5" t="n"/>
       <c r="K26" s="5" t="n">
-        <v>1.11</v>
+        <v>1.07</v>
       </c>
       <c r="L26" s="5" t="n">
         <v>1.46</v>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Hands where all cards are on an edge score +15 pips per card</t>
+          <t>Cards scored on an edge score +15 pips</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2076,13 +2076,13 @@
         <v/>
       </c>
       <c r="K27" s="5" t="n">
-        <v>0.61</v>
+        <v>1.94</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>1.25</v>
+        <v>1.82</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
@@ -2093,7 +2093,7 @@
       <c r="P27" s="7" t="inlineStr"/>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>Hands where all cards are on an edge score +{pips_per_card} pips per card</t>
+          <t>Cards scored on an edge score +{pips_per_card} pips</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -2145,7 +2145,7 @@
         <v/>
       </c>
       <c r="K28" s="5" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="L28" s="5" t="n">
         <v>1.13</v>
@@ -2214,7 +2214,7 @@
         <v/>
       </c>
       <c r="K29" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.66</v>
       </c>
       <c r="L29" s="5" t="n">
         <v>1.28</v>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr"/>
@@ -2283,10 +2283,10 @@
         <v/>
       </c>
       <c r="K30" s="5" t="n">
-        <v>3.06</v>
+        <v>3.19</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>2.26</v>
+        <v>2.35</v>
       </c>
       <c r="M30" s="6" t="n">
         <v>84</v>
@@ -2815,10 +2815,10 @@
         <v/>
       </c>
       <c r="K41" s="5" t="n">
-        <v>2.79</v>
+        <v>2.68</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>2.15</v>
+        <v>2.14</v>
       </c>
       <c r="M41" s="6" t="n">
         <v>100</v>
@@ -2943,7 +2943,7 @@
         <v/>
       </c>
       <c r="K43" s="5" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="L43" s="5" t="n">
         <v>1.13</v>
@@ -3012,7 +3012,7 @@
         <v/>
       </c>
       <c r="K44" s="5" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="L44" s="5" t="n">
         <v>1.34</v>
@@ -3077,7 +3077,7 @@
         <v/>
       </c>
       <c r="K45" s="5" t="n">
-        <v>1.07</v>
+        <v>1.04</v>
       </c>
       <c r="L45" s="5" t="n">
         <v>1.44</v>
@@ -3142,7 +3142,7 @@
         <v/>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1.62</v>
+        <v>1.57</v>
       </c>
       <c r="L46" s="5" t="n">
         <v>1.67</v>
@@ -3207,7 +3207,7 @@
         <v/>
       </c>
       <c r="K47" s="5" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="L47" s="5" t="n">
         <v>1.17</v>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="N47" s="3" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr"/>
@@ -3262,7 +3262,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>Build: 2026-10-20 · r606 · Double-tap a marked challenge cell to bring it now; double-tap the clock skull to skip to the boss</t>
+          <t>Build: 2026-10-21 · r619 · Trick tour (?tricks): the common Tricks one by one with their numbers live; the Trick balance sheet</t>
         </is>
       </c>
     </row>

</xml_diff>